<commit_message>
chore(infra): institutionalize CIE research engine v1.0.0
- Canonical Ingestion: Consolidated 3-pillar engine (world_bank, http_api, local_file).
- Smart Intelligence: Implemented agnostic loading ladder and automated path resolution.
- Quality Hardening: Resolved 29 ruff errors and aligned with PE8 standards.
- Governance: Hardened .gitignore to protect researchers' landing zone and exclude >100MB binaries.
- Documentation: Established institutional-grade manual and technical architecture.
- Testing: Validated infrastructure contract with 100% test pass (active suite).
</commit_message>
<xml_diff>
--- a/data/raw/excel/Base_Raw_Ecuador_Homicidios_Long.xlsx
+++ b/data/raw/excel/Base_Raw_Ecuador_Homicidios_Long.xlsx
@@ -15,7 +15,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="106" uniqueCount="33">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="118" uniqueCount="37">
   <si>
     <t>Variables</t>
   </si>
@@ -29,6 +29,12 @@
     <t>Fuente</t>
   </si>
   <si>
+    <t>Backend</t>
+  </si>
+  <si>
+    <t>Alcance</t>
+  </si>
+  <si>
     <t>Link</t>
   </si>
   <si>
@@ -84,6 +90,12 @@
   </si>
   <si>
     <t>SIPRI</t>
+  </si>
+  <si>
+    <t>world_bank</t>
+  </si>
+  <si>
+    <t>global</t>
   </si>
   <si>
     <t>https://data.worldbank.org/indicator/VC.IHR.PSRC.P5</t>
@@ -458,13 +470,13 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:E6"/>
+  <dimension ref="A1:G6"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="1" max="26" width="22.7109375" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:5">
+    <row r="1" spans="1:7">
       <c r="A1" t="s">
         <v>0</v>
       </c>
@@ -480,99 +492,135 @@
       <c r="E1" t="s">
         <v>4</v>
       </c>
-    </row>
-    <row r="2" spans="1:5">
+      <c r="F1" t="s">
+        <v>5</v>
+      </c>
+      <c r="G1" t="s">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="2" spans="1:7">
       <c r="A2" t="s">
-        <v>5</v>
+        <v>7</v>
       </c>
       <c r="B2" t="s">
+        <v>12</v>
+      </c>
+      <c r="C2" t="s">
+        <v>16</v>
+      </c>
+      <c r="D2" t="s">
+        <v>21</v>
+      </c>
+      <c r="E2" t="s">
+        <v>25</v>
+      </c>
+      <c r="F2" t="s">
+        <v>26</v>
+      </c>
+      <c r="G2" s="1" t="s">
+        <v>27</v>
+      </c>
+    </row>
+    <row r="3" spans="1:7">
+      <c r="A3" t="s">
+        <v>8</v>
+      </c>
+      <c r="B3" t="s">
+        <v>13</v>
+      </c>
+      <c r="C3" t="s">
+        <v>17</v>
+      </c>
+      <c r="D3" t="s">
+        <v>22</v>
+      </c>
+      <c r="E3" t="s">
+        <v>25</v>
+      </c>
+      <c r="F3" t="s">
+        <v>26</v>
+      </c>
+      <c r="G3" s="1" t="s">
+        <v>28</v>
+      </c>
+    </row>
+    <row r="4" spans="1:7">
+      <c r="A4" t="s">
+        <v>9</v>
+      </c>
+      <c r="B4" t="s">
+        <v>14</v>
+      </c>
+      <c r="C4" t="s">
+        <v>18</v>
+      </c>
+      <c r="D4" t="s">
+        <v>23</v>
+      </c>
+      <c r="E4" t="s">
+        <v>25</v>
+      </c>
+      <c r="F4" t="s">
+        <v>26</v>
+      </c>
+      <c r="G4" s="1" t="s">
+        <v>29</v>
+      </c>
+    </row>
+    <row r="5" spans="1:7">
+      <c r="A5" t="s">
         <v>10</v>
       </c>
-      <c r="C2" t="s">
-        <v>14</v>
-      </c>
-      <c r="D2" t="s">
+      <c r="B5" t="s">
+        <v>15</v>
+      </c>
+      <c r="C5" t="s">
         <v>19</v>
       </c>
-      <c r="E2" s="1" t="s">
+      <c r="D5" t="s">
+        <v>24</v>
+      </c>
+      <c r="E5" t="s">
+        <v>25</v>
+      </c>
+      <c r="F5" t="s">
+        <v>26</v>
+      </c>
+      <c r="G5" s="1" t="s">
+        <v>30</v>
+      </c>
+    </row>
+    <row r="6" spans="1:7">
+      <c r="A6" t="s">
+        <v>11</v>
+      </c>
+      <c r="B6" t="s">
+        <v>15</v>
+      </c>
+      <c r="C6" t="s">
+        <v>20</v>
+      </c>
+      <c r="D6" t="s">
         <v>23</v>
       </c>
-    </row>
-    <row r="3" spans="1:5">
-      <c r="A3" t="s">
-        <v>6</v>
-      </c>
-      <c r="B3" t="s">
-        <v>11</v>
-      </c>
-      <c r="C3" t="s">
-        <v>15</v>
-      </c>
-      <c r="D3" t="s">
-        <v>20</v>
-      </c>
-      <c r="E3" s="1" t="s">
-        <v>24</v>
-      </c>
-    </row>
-    <row r="4" spans="1:5">
-      <c r="A4" t="s">
-        <v>7</v>
-      </c>
-      <c r="B4" t="s">
-        <v>12</v>
-      </c>
-      <c r="C4" t="s">
-        <v>16</v>
-      </c>
-      <c r="D4" t="s">
-        <v>21</v>
-      </c>
-      <c r="E4" s="1" t="s">
+      <c r="E6" t="s">
         <v>25</v>
       </c>
-    </row>
-    <row r="5" spans="1:5">
-      <c r="A5" t="s">
-        <v>8</v>
-      </c>
-      <c r="B5" t="s">
-        <v>13</v>
-      </c>
-      <c r="C5" t="s">
-        <v>17</v>
-      </c>
-      <c r="D5" t="s">
-        <v>22</v>
-      </c>
-      <c r="E5" s="1" t="s">
+      <c r="F6" t="s">
         <v>26</v>
       </c>
-    </row>
-    <row r="6" spans="1:5">
-      <c r="A6" t="s">
-        <v>9</v>
-      </c>
-      <c r="B6" t="s">
-        <v>13</v>
-      </c>
-      <c r="C6" t="s">
-        <v>18</v>
-      </c>
-      <c r="D6" t="s">
-        <v>21</v>
-      </c>
-      <c r="E6" s="1" t="s">
-        <v>27</v>
+      <c r="G6" s="1" t="s">
+        <v>31</v>
       </c>
     </row>
   </sheetData>
   <hyperlinks>
-    <hyperlink ref="E2" r:id="rId1"/>
-    <hyperlink ref="E3" r:id="rId2"/>
-    <hyperlink ref="E4" r:id="rId3"/>
-    <hyperlink ref="E5" r:id="rId4"/>
-    <hyperlink ref="E6" r:id="rId5"/>
+    <hyperlink ref="G2" r:id="rId1"/>
+    <hyperlink ref="G3" r:id="rId2"/>
+    <hyperlink ref="G4" r:id="rId3"/>
+    <hyperlink ref="G5" r:id="rId4"/>
+    <hyperlink ref="G6" r:id="rId5"/>
   </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
@@ -588,36 +636,36 @@
   <sheetData>
     <row r="1" spans="1:8">
       <c r="A1" t="s">
-        <v>28</v>
+        <v>32</v>
       </c>
       <c r="B1" t="s">
-        <v>29</v>
+        <v>33</v>
       </c>
       <c r="C1" t="s">
-        <v>30</v>
+        <v>34</v>
       </c>
       <c r="D1" t="s">
-        <v>5</v>
+        <v>7</v>
       </c>
       <c r="E1" t="s">
-        <v>6</v>
+        <v>8</v>
       </c>
       <c r="F1" t="s">
-        <v>7</v>
+        <v>9</v>
       </c>
       <c r="G1" t="s">
-        <v>8</v>
+        <v>10</v>
       </c>
       <c r="H1" t="s">
-        <v>9</v>
+        <v>11</v>
       </c>
     </row>
     <row r="2" spans="1:8">
       <c r="A2" t="s">
-        <v>31</v>
+        <v>35</v>
       </c>
       <c r="B2" t="s">
-        <v>32</v>
+        <v>36</v>
       </c>
       <c r="C2">
         <v>1990</v>
@@ -628,6 +676,9 @@
       <c r="E2">
         <v>5.881</v>
       </c>
+      <c r="F2">
+        <v>0</v>
+      </c>
       <c r="G2">
         <v>1.35122222907748</v>
       </c>
@@ -637,10 +688,10 @@
     </row>
     <row r="3" spans="1:8">
       <c r="A3" t="s">
-        <v>31</v>
+        <v>35</v>
       </c>
       <c r="B3" t="s">
-        <v>32</v>
+        <v>36</v>
       </c>
       <c r="C3">
         <v>1991</v>
@@ -663,10 +714,10 @@
     </row>
     <row r="4" spans="1:8">
       <c r="A4" t="s">
-        <v>31</v>
+        <v>35</v>
       </c>
       <c r="B4" t="s">
-        <v>32</v>
+        <v>36</v>
       </c>
       <c r="C4">
         <v>1992</v>
@@ -677,6 +728,9 @@
       <c r="E4">
         <v>8.56</v>
       </c>
+      <c r="F4">
+        <v>0.00512</v>
+      </c>
       <c r="G4">
         <v>1.21330539339896</v>
       </c>
@@ -686,10 +740,10 @@
     </row>
     <row r="5" spans="1:8">
       <c r="A5" t="s">
-        <v>31</v>
+        <v>35</v>
       </c>
       <c r="B5" t="s">
-        <v>32</v>
+        <v>36</v>
       </c>
       <c r="C5">
         <v>1993</v>
@@ -700,6 +754,9 @@
       <c r="E5">
         <v>7.948</v>
       </c>
+      <c r="F5">
+        <v>0.0164</v>
+      </c>
       <c r="G5">
         <v>1.5053435537415</v>
       </c>
@@ -709,10 +766,10 @@
     </row>
     <row r="6" spans="1:8">
       <c r="A6" t="s">
-        <v>31</v>
+        <v>35</v>
       </c>
       <c r="B6" t="s">
-        <v>32</v>
+        <v>36</v>
       </c>
       <c r="C6">
         <v>1994</v>
@@ -723,6 +780,9 @@
       <c r="E6">
         <v>6.68</v>
       </c>
+      <c r="F6">
+        <v>0.0348</v>
+      </c>
       <c r="G6">
         <v>1.31569135777556</v>
       </c>
@@ -732,10 +792,10 @@
     </row>
     <row r="7" spans="1:8">
       <c r="A7" t="s">
-        <v>31</v>
+        <v>35</v>
       </c>
       <c r="B7" t="s">
-        <v>32</v>
+        <v>36</v>
       </c>
       <c r="C7">
         <v>1995</v>
@@ -746,6 +806,9 @@
       <c r="E7">
         <v>6.701</v>
       </c>
+      <c r="F7">
+        <v>0.0438</v>
+      </c>
       <c r="G7">
         <v>1.98760353101763</v>
       </c>
@@ -755,10 +818,10 @@
     </row>
     <row r="8" spans="1:8">
       <c r="A8" t="s">
-        <v>31</v>
+        <v>35</v>
       </c>
       <c r="B8" t="s">
-        <v>32</v>
+        <v>36</v>
       </c>
       <c r="C8">
         <v>1996</v>
@@ -769,6 +832,9 @@
       <c r="E8">
         <v>10.376</v>
       </c>
+      <c r="F8">
+        <v>0.0862</v>
+      </c>
       <c r="G8">
         <v>1.6897249235818</v>
       </c>
@@ -778,10 +844,10 @@
     </row>
     <row r="9" spans="1:8">
       <c r="A9" t="s">
-        <v>31</v>
+        <v>35</v>
       </c>
       <c r="B9" t="s">
-        <v>32</v>
+        <v>36</v>
       </c>
       <c r="C9">
         <v>1997</v>
@@ -792,6 +858,9 @@
       <c r="E9">
         <v>9.169</v>
       </c>
+      <c r="F9">
+        <v>0.11</v>
+      </c>
       <c r="G9">
         <v>1.8110665611487</v>
       </c>
@@ -801,10 +870,10 @@
     </row>
     <row r="10" spans="1:8">
       <c r="A10" t="s">
-        <v>31</v>
+        <v>35</v>
       </c>
       <c r="B10" t="s">
-        <v>32</v>
+        <v>36</v>
       </c>
       <c r="C10">
         <v>1998</v>
@@ -815,6 +884,9 @@
       <c r="E10">
         <v>11.492</v>
       </c>
+      <c r="F10">
+        <v>0.125</v>
+      </c>
       <c r="G10">
         <v>2.01895367462851</v>
       </c>
@@ -824,10 +896,10 @@
     </row>
     <row r="11" spans="1:8">
       <c r="A11" t="s">
-        <v>31</v>
+        <v>35</v>
       </c>
       <c r="B11" t="s">
-        <v>32</v>
+        <v>36</v>
       </c>
       <c r="C11">
         <v>1999</v>
@@ -838,6 +910,9 @@
       <c r="E11">
         <v>13.961</v>
       </c>
+      <c r="F11">
+        <v>0.823</v>
+      </c>
       <c r="G11">
         <v>1.55598240646013</v>
       </c>
@@ -847,10 +922,10 @@
     </row>
     <row r="12" spans="1:8">
       <c r="A12" t="s">
-        <v>31</v>
+        <v>35</v>
       </c>
       <c r="B12" t="s">
-        <v>32</v>
+        <v>36</v>
       </c>
       <c r="C12">
         <v>2000</v>
@@ -861,6 +936,9 @@
       <c r="E12">
         <v>4.8</v>
       </c>
+      <c r="F12">
+        <v>1.46218853556457</v>
+      </c>
       <c r="G12">
         <v>1.51733948117752</v>
       </c>
@@ -870,10 +948,10 @@
     </row>
     <row r="13" spans="1:8">
       <c r="A13" t="s">
-        <v>31</v>
+        <v>35</v>
       </c>
       <c r="B13" t="s">
-        <v>32</v>
+        <v>36</v>
       </c>
       <c r="C13">
         <v>2001</v>
@@ -884,6 +962,9 @@
       <c r="E13">
         <v>4.252</v>
       </c>
+      <c r="F13">
+        <v>2.67044367376705</v>
+      </c>
       <c r="G13">
         <v>1.66039298461832</v>
       </c>
@@ -893,10 +974,10 @@
     </row>
     <row r="14" spans="1:8">
       <c r="A14" t="s">
-        <v>31</v>
+        <v>35</v>
       </c>
       <c r="B14" t="s">
-        <v>32</v>
+        <v>36</v>
       </c>
       <c r="C14">
         <v>2002</v>
@@ -907,6 +988,9 @@
       <c r="E14">
         <v>7.168</v>
       </c>
+      <c r="F14">
+        <v>4.26079691519764</v>
+      </c>
       <c r="G14">
         <v>1.86662346180863</v>
       </c>
@@ -916,10 +1000,10 @@
     </row>
     <row r="15" spans="1:8">
       <c r="A15" t="s">
-        <v>31</v>
+        <v>35</v>
       </c>
       <c r="B15" t="s">
-        <v>32</v>
+        <v>36</v>
       </c>
       <c r="C15">
         <v>2003</v>
@@ -930,6 +1014,9 @@
       <c r="E15">
         <v>5.662</v>
       </c>
+      <c r="F15">
+        <v>4.46022834472698</v>
+      </c>
       <c r="G15">
         <v>2.38654946619875</v>
       </c>
@@ -939,10 +1026,10 @@
     </row>
     <row r="16" spans="1:8">
       <c r="A16" t="s">
-        <v>31</v>
+        <v>35</v>
       </c>
       <c r="B16" t="s">
-        <v>32</v>
+        <v>36</v>
       </c>
       <c r="C16">
         <v>2004</v>
@@ -953,6 +1040,9 @@
       <c r="E16">
         <v>5.002</v>
       </c>
+      <c r="F16">
+        <v>4.83444263759525</v>
+      </c>
       <c r="G16">
         <v>2.01733501271599</v>
       </c>
@@ -962,10 +1052,10 @@
     </row>
     <row r="17" spans="1:8">
       <c r="A17" t="s">
-        <v>31</v>
+        <v>35</v>
       </c>
       <c r="B17" t="s">
-        <v>32</v>
+        <v>36</v>
       </c>
       <c r="C17">
         <v>2005</v>
@@ -976,6 +1066,9 @@
       <c r="E17">
         <v>3.779</v>
       </c>
+      <c r="F17">
+        <v>5.994299889</v>
+      </c>
       <c r="G17">
         <v>2.36848865849083</v>
       </c>
@@ -985,10 +1078,10 @@
     </row>
     <row r="18" spans="1:8">
       <c r="A18" t="s">
-        <v>31</v>
+        <v>35</v>
       </c>
       <c r="B18" t="s">
-        <v>32</v>
+        <v>36</v>
       </c>
       <c r="C18">
         <v>2006</v>
@@ -999,6 +1092,9 @@
       <c r="E18">
         <v>3.55</v>
       </c>
+      <c r="F18">
+        <v>7.199999809</v>
+      </c>
       <c r="G18">
         <v>2.07919490158198</v>
       </c>
@@ -1008,10 +1104,10 @@
     </row>
     <row r="19" spans="1:8">
       <c r="A19" t="s">
-        <v>31</v>
+        <v>35</v>
       </c>
       <c r="B19" t="s">
-        <v>32</v>
+        <v>36</v>
       </c>
       <c r="C19">
         <v>2007</v>
@@ -1022,6 +1118,9 @@
       <c r="E19">
         <v>3.142</v>
       </c>
+      <c r="F19">
+        <v>10.80000019</v>
+      </c>
       <c r="G19">
         <v>2.62795079870115</v>
       </c>
@@ -1031,10 +1130,10 @@
     </row>
     <row r="20" spans="1:8">
       <c r="A20" t="s">
-        <v>31</v>
+        <v>35</v>
       </c>
       <c r="B20" t="s">
-        <v>32</v>
+        <v>36</v>
       </c>
       <c r="C20">
         <v>2008</v>
@@ -1045,6 +1144,9 @@
       <c r="E20">
         <v>3.917</v>
       </c>
+      <c r="F20">
+        <v>18.8</v>
+      </c>
       <c r="G20">
         <v>2.6922066648737</v>
       </c>
@@ -1054,10 +1156,10 @@
     </row>
     <row r="21" spans="1:8">
       <c r="A21" t="s">
-        <v>31</v>
+        <v>35</v>
       </c>
       <c r="B21" t="s">
-        <v>32</v>
+        <v>36</v>
       </c>
       <c r="C21">
         <v>2009</v>
@@ -1068,6 +1170,9 @@
       <c r="E21">
         <v>4.608</v>
       </c>
+      <c r="F21">
+        <v>24.6</v>
+      </c>
       <c r="G21">
         <v>3.24319951406484</v>
       </c>
@@ -1077,10 +1182,10 @@
     </row>
     <row r="22" spans="1:8">
       <c r="A22" t="s">
-        <v>31</v>
+        <v>35</v>
       </c>
       <c r="B22" t="s">
-        <v>32</v>
+        <v>36</v>
       </c>
       <c r="C22">
         <v>2010</v>
@@ -1091,6 +1196,9 @@
       <c r="E22">
         <v>4.088</v>
       </c>
+      <c r="F22">
+        <v>29.03</v>
+      </c>
       <c r="G22">
         <v>3.07257396611835</v>
       </c>
@@ -1100,10 +1208,10 @@
     </row>
     <row r="23" spans="1:8">
       <c r="A23" t="s">
-        <v>31</v>
+        <v>35</v>
       </c>
       <c r="B23" t="s">
-        <v>32</v>
+        <v>36</v>
       </c>
       <c r="C23">
         <v>2011</v>
@@ -1114,6 +1222,9 @@
       <c r="E23">
         <v>3.458</v>
       </c>
+      <c r="F23">
+        <v>31.3668083587433</v>
+      </c>
       <c r="G23">
         <v>3.10647440690889</v>
       </c>
@@ -1123,10 +1234,10 @@
     </row>
     <row r="24" spans="1:8">
       <c r="A24" t="s">
-        <v>31</v>
+        <v>35</v>
       </c>
       <c r="B24" t="s">
-        <v>32</v>
+        <v>36</v>
       </c>
       <c r="C24">
         <v>2012</v>
@@ -1137,6 +1248,9 @@
       <c r="E24">
         <v>3.235</v>
       </c>
+      <c r="F24">
+        <v>35.1351464545516</v>
+      </c>
       <c r="G24">
         <v>2.95181465866835</v>
       </c>
@@ -1146,10 +1260,10 @@
     </row>
     <row r="25" spans="1:8">
       <c r="A25" t="s">
-        <v>31</v>
+        <v>35</v>
       </c>
       <c r="B25" t="s">
-        <v>32</v>
+        <v>36</v>
       </c>
       <c r="C25">
         <v>2013</v>
@@ -1160,6 +1274,9 @@
       <c r="E25">
         <v>2.913</v>
       </c>
+      <c r="F25">
+        <v>40.279121941</v>
+      </c>
       <c r="G25">
         <v>2.83298697009902</v>
       </c>
@@ -1169,10 +1286,10 @@
     </row>
     <row r="26" spans="1:8">
       <c r="A26" t="s">
-        <v>31</v>
+        <v>35</v>
       </c>
       <c r="B26" t="s">
-        <v>32</v>
+        <v>36</v>
       </c>
       <c r="C26">
         <v>2014</v>
@@ -1183,6 +1300,9 @@
       <c r="E26">
         <v>3.279</v>
       </c>
+      <c r="F26">
+        <v>45.5903906666095</v>
+      </c>
       <c r="G26">
         <v>2.71279094772759</v>
       </c>
@@ -1192,10 +1312,10 @@
     </row>
     <row r="27" spans="1:8">
       <c r="A27" t="s">
-        <v>31</v>
+        <v>35</v>
       </c>
       <c r="B27" t="s">
-        <v>32</v>
+        <v>36</v>
       </c>
       <c r="C27">
         <v>2015</v>
@@ -1206,6 +1326,9 @@
       <c r="E27">
         <v>3.419</v>
       </c>
+      <c r="F27">
+        <v>48.9404337892669</v>
+      </c>
       <c r="G27">
         <v>2.6720726618256</v>
       </c>
@@ -1215,10 +1338,10 @@
     </row>
     <row r="28" spans="1:8">
       <c r="A28" t="s">
-        <v>31</v>
+        <v>35</v>
       </c>
       <c r="B28" t="s">
-        <v>32</v>
+        <v>36</v>
       </c>
       <c r="C28">
         <v>2016</v>
@@ -1229,6 +1352,9 @@
       <c r="E28">
         <v>4.39</v>
       </c>
+      <c r="F28">
+        <v>54.0629247288864</v>
+      </c>
       <c r="G28">
         <v>2.57311675623471</v>
       </c>
@@ -1238,10 +1364,10 @@
     </row>
     <row r="29" spans="1:8">
       <c r="A29" t="s">
-        <v>31</v>
+        <v>35</v>
       </c>
       <c r="B29" t="s">
-        <v>32</v>
+        <v>36</v>
       </c>
       <c r="C29">
         <v>2017</v>
@@ -1252,6 +1378,9 @@
       <c r="E29">
         <v>3.708</v>
       </c>
+      <c r="F29">
+        <v>55.79999924</v>
+      </c>
       <c r="G29">
         <v>2.35738419773924</v>
       </c>
@@ -1261,10 +1390,10 @@
     </row>
     <row r="30" spans="1:8">
       <c r="A30" t="s">
-        <v>31</v>
+        <v>35</v>
       </c>
       <c r="B30" t="s">
-        <v>32</v>
+        <v>36</v>
       </c>
       <c r="C30">
         <v>2018</v>
@@ -1275,6 +1404,9 @@
       <c r="E30">
         <v>3.396</v>
       </c>
+      <c r="F30">
+        <v>57.5</v>
+      </c>
       <c r="G30">
         <v>2.37199911152844</v>
       </c>
@@ -1284,10 +1416,10 @@
     </row>
     <row r="31" spans="1:8">
       <c r="A31" t="s">
-        <v>31</v>
+        <v>35</v>
       </c>
       <c r="B31" t="s">
-        <v>32</v>
+        <v>36</v>
       </c>
       <c r="C31">
         <v>2019</v>
@@ -1298,6 +1430,9 @@
       <c r="E31">
         <v>3.703</v>
       </c>
+      <c r="F31">
+        <v>59.2</v>
+      </c>
       <c r="G31">
         <v>2.18038189769994</v>
       </c>
@@ -1307,10 +1442,10 @@
     </row>
     <row r="32" spans="1:8">
       <c r="A32" t="s">
-        <v>31</v>
+        <v>35</v>
       </c>
       <c r="B32" t="s">
-        <v>32</v>
+        <v>36</v>
       </c>
       <c r="C32">
         <v>2020</v>
@@ -1321,6 +1456,9 @@
       <c r="E32">
         <v>6.084</v>
       </c>
+      <c r="F32">
+        <v>70.7</v>
+      </c>
       <c r="G32">
         <v>2.45792351121034</v>
       </c>
@@ -1330,10 +1468,10 @@
     </row>
     <row r="33" spans="1:8">
       <c r="A33" t="s">
-        <v>31</v>
+        <v>35</v>
       </c>
       <c r="B33" t="s">
-        <v>32</v>
+        <v>36</v>
       </c>
       <c r="C33">
         <v>2021</v>
@@ -1344,6 +1482,9 @@
       <c r="E33">
         <v>4.434</v>
       </c>
+      <c r="F33">
+        <v>69.1147995</v>
+      </c>
       <c r="G33">
         <v>2.24210709535338</v>
       </c>
@@ -1353,10 +1494,10 @@
     </row>
     <row r="34" spans="1:8">
       <c r="A34" t="s">
-        <v>31</v>
+        <v>35</v>
       </c>
       <c r="B34" t="s">
-        <v>32</v>
+        <v>36</v>
       </c>
       <c r="C34">
         <v>2022</v>
@@ -1367,6 +1508,9 @@
       <c r="E34">
         <v>3.672</v>
       </c>
+      <c r="F34">
+        <v>69.71811356000001</v>
+      </c>
       <c r="G34">
         <v>2.21851529975547</v>
       </c>
@@ -1376,10 +1520,10 @@
     </row>
     <row r="35" spans="1:8">
       <c r="A35" t="s">
-        <v>31</v>
+        <v>35</v>
       </c>
       <c r="B35" t="s">
-        <v>32</v>
+        <v>36</v>
       </c>
       <c r="C35">
         <v>2023</v>
@@ -1389,6 +1533,9 @@
       </c>
       <c r="E35">
         <v>3.462</v>
+      </c>
+      <c r="F35">
+        <v>72.6943146</v>
       </c>
       <c r="G35">
         <v>2.2651385614971</v>

</xml_diff>